<commit_message>
Miyawaki nord-est: aleea în buclă largă în jurul luminișului în locul cârligului; traversările aleii cu tub orb la irigare; toate derivatele regenerate
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/cereri/cerere-oferta-pepiniera-foresta-srl.xlsx
+++ b/resurse/oferte/cereri/cerere-oferta-pepiniera-foresta-srl.xlsx
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="D12" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="D13" s="5" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="D15" s="5" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="D18" s="5" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>

</xml_diff>